<commit_message>
Enhance spreadsheet with non-monthly expenses sheet and improved projection
Co-authored-by: whitbeck <251054+whitbeck@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Account_Balance_Tracker.xlsx
+++ b/Account_Balance_Tracker.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Configuration" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Projection" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Expense History" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Non-Monthly Expenses" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -55,7 +56,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -66,6 +67,30 @@
       <patternFill patternType="solid">
         <fgColor rgb="004472C4"/>
         <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0070AD47"/>
+        <bgColor rgb="0070AD47"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+        <bgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -81,7 +106,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -94,10 +119,19 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -551,19 +585,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J35"/>
+  <dimension ref="A1:L50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -583,7 +619,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>Add one-time expenses in the 'Other Expenses' column.</t>
+          <t>Add one-time expenses in the 'Other Expenses' column. Non-monthly expenses appear in their own column.</t>
         </is>
       </c>
     </row>
@@ -625,15 +661,25 @@
       </c>
       <c r="H5" s="8" t="inlineStr">
         <is>
+          <t>Non-Monthly</t>
+        </is>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
           <t>Other Expenses</t>
         </is>
       </c>
-      <c r="I5" s="8" t="inlineStr">
+      <c r="J5" s="8" t="inlineStr">
+        <is>
+          <t>Total Recurring</t>
+        </is>
+      </c>
+      <c r="K5" s="8" t="inlineStr">
         <is>
           <t>Total Expenses</t>
         </is>
       </c>
-      <c r="J5" s="8" t="inlineStr">
+      <c r="L5" s="8" t="inlineStr">
         <is>
           <t>Balance</t>
         </is>
@@ -649,7 +695,7 @@
         <f>Configuration!B4</f>
         <v/>
       </c>
-      <c r="J6" s="9">
+      <c r="L6" s="9">
         <f>Configuration!B3</f>
         <v/>
       </c>
@@ -678,15 +724,22 @@
       <c r="G7" s="3" t="n">
         <v>80</v>
       </c>
-      <c r="H7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="3">
-        <f>SUM(D7:H7)</f>
-        <v/>
-      </c>
-      <c r="J7" s="9">
-        <f>J6+C7-I7</f>
+      <c r="H7" s="10" t="n">
+        <v>750</v>
+      </c>
+      <c r="I7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="3">
+        <f>SUM(D7:G7)</f>
+        <v/>
+      </c>
+      <c r="K7" s="9">
+        <f>SUM(D7:I7)</f>
+        <v/>
+      </c>
+      <c r="L7" s="9">
+        <f>L6+C7-K7</f>
         <v/>
       </c>
     </row>
@@ -714,51 +767,65 @@
       <c r="G8" s="3" t="n">
         <v>80</v>
       </c>
-      <c r="H8" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="3">
-        <f>SUM(D8:H8)</f>
-        <v/>
-      </c>
-      <c r="J8" s="9">
-        <f>J7+C8-I8</f>
+      <c r="H8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="3">
+        <f>SUM(D8:G8)</f>
+        <v/>
+      </c>
+      <c r="K8" s="9">
+        <f>SUM(D8:I8)</f>
+        <v/>
+      </c>
+      <c r="L8" s="9">
+        <f>L7+C8-K8</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="B9" s="4">
+      <c r="B9" s="13">
         <f>DATE(YEAR(B6), MONTH(B6)+3, 1)</f>
         <v/>
       </c>
-      <c r="C9" s="3">
-        <f>Configuration!B7*2</f>
-        <v/>
-      </c>
-      <c r="D9" s="3" t="n">
+      <c r="C9" s="14">
+        <f>Configuration!B7*2</f>
+        <v/>
+      </c>
+      <c r="D9" s="14" t="n">
         <v>350</v>
       </c>
-      <c r="E9" s="3" t="n">
-        <v>250</v>
-      </c>
-      <c r="F9" s="3" t="n">
+      <c r="E9" s="14" t="n">
+        <v>250</v>
+      </c>
+      <c r="F9" s="14" t="n">
         <v>160</v>
       </c>
-      <c r="G9" s="3" t="n">
+      <c r="G9" s="14" t="n">
         <v>80</v>
       </c>
-      <c r="H9" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="3">
-        <f>SUM(D9:H9)</f>
-        <v/>
-      </c>
-      <c r="J9" s="9">
-        <f>J8+C9-I9</f>
+      <c r="H9" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="14">
+        <f>SUM(D9:G9)</f>
+        <v/>
+      </c>
+      <c r="K9" s="15">
+        <f>SUM(D9:I9)</f>
+        <v/>
+      </c>
+      <c r="L9" s="15">
+        <f>L8+C9-K9</f>
         <v/>
       </c>
     </row>
@@ -786,15 +853,22 @@
       <c r="G10" s="3" t="n">
         <v>80</v>
       </c>
-      <c r="H10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="3">
-        <f>SUM(D10:H10)</f>
-        <v/>
-      </c>
-      <c r="J10" s="9">
-        <f>J9+C10-I10</f>
+      <c r="H10" s="10" t="n">
+        <v>2550</v>
+      </c>
+      <c r="I10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="3">
+        <f>SUM(D10:G10)</f>
+        <v/>
+      </c>
+      <c r="K10" s="9">
+        <f>SUM(D10:I10)</f>
+        <v/>
+      </c>
+      <c r="L10" s="9">
+        <f>L9+C10-K10</f>
         <v/>
       </c>
     </row>
@@ -822,51 +896,65 @@
       <c r="G11" s="3" t="n">
         <v>80</v>
       </c>
-      <c r="H11" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="3">
-        <f>SUM(D11:H11)</f>
-        <v/>
-      </c>
-      <c r="J11" s="9">
-        <f>J10+C11-I11</f>
+      <c r="H11" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="3">
+        <f>SUM(D11:G11)</f>
+        <v/>
+      </c>
+      <c r="K11" s="9">
+        <f>SUM(D11:I11)</f>
+        <v/>
+      </c>
+      <c r="L11" s="9">
+        <f>L10+C11-K11</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
+      <c r="A12" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="B12" s="4">
+      <c r="B12" s="13">
         <f>DATE(YEAR(B6), MONTH(B6)+6, 1)</f>
         <v/>
       </c>
-      <c r="C12" s="3">
-        <f>Configuration!B7*2</f>
-        <v/>
-      </c>
-      <c r="D12" s="3" t="n">
+      <c r="C12" s="14">
+        <f>Configuration!B7*2</f>
+        <v/>
+      </c>
+      <c r="D12" s="14" t="n">
         <v>350</v>
       </c>
-      <c r="E12" s="3" t="n">
-        <v>250</v>
-      </c>
-      <c r="F12" s="3" t="n">
+      <c r="E12" s="14" t="n">
+        <v>250</v>
+      </c>
+      <c r="F12" s="14" t="n">
         <v>160</v>
       </c>
-      <c r="G12" s="3" t="n">
+      <c r="G12" s="14" t="n">
         <v>80</v>
       </c>
-      <c r="H12" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="3">
-        <f>SUM(D12:H12)</f>
-        <v/>
-      </c>
-      <c r="J12" s="9">
-        <f>J11+C12-I12</f>
+      <c r="H12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="14">
+        <f>SUM(D12:G12)</f>
+        <v/>
+      </c>
+      <c r="K12" s="15">
+        <f>SUM(D12:I12)</f>
+        <v/>
+      </c>
+      <c r="L12" s="15">
+        <f>L11+C12-K12</f>
         <v/>
       </c>
     </row>
@@ -894,15 +982,22 @@
       <c r="G13" s="3" t="n">
         <v>80</v>
       </c>
-      <c r="H13" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="3">
-        <f>SUM(D13:H13)</f>
-        <v/>
-      </c>
-      <c r="J13" s="9">
-        <f>J12+C13-I13</f>
+      <c r="H13" s="10" t="n">
+        <v>750</v>
+      </c>
+      <c r="I13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="3">
+        <f>SUM(D13:G13)</f>
+        <v/>
+      </c>
+      <c r="K13" s="9">
+        <f>SUM(D13:I13)</f>
+        <v/>
+      </c>
+      <c r="L13" s="9">
+        <f>L12+C13-K13</f>
         <v/>
       </c>
     </row>
@@ -930,51 +1025,65 @@
       <c r="G14" s="3" t="n">
         <v>80</v>
       </c>
-      <c r="H14" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="3">
-        <f>SUM(D14:H14)</f>
-        <v/>
-      </c>
-      <c r="J14" s="9">
-        <f>J13+C14-I14</f>
+      <c r="H14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="3">
+        <f>SUM(D14:G14)</f>
+        <v/>
+      </c>
+      <c r="K14" s="9">
+        <f>SUM(D14:I14)</f>
+        <v/>
+      </c>
+      <c r="L14" s="9">
+        <f>L13+C14-K14</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="n">
+      <c r="A15" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="B15" s="4">
+      <c r="B15" s="13">
         <f>DATE(YEAR(B6), MONTH(B6)+9, 1)</f>
         <v/>
       </c>
-      <c r="C15" s="3">
-        <f>Configuration!B7*2</f>
-        <v/>
-      </c>
-      <c r="D15" s="3" t="n">
+      <c r="C15" s="14">
+        <f>Configuration!B7*2</f>
+        <v/>
+      </c>
+      <c r="D15" s="14" t="n">
         <v>280</v>
       </c>
-      <c r="E15" s="3" t="n">
-        <v>250</v>
-      </c>
-      <c r="F15" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" s="3" t="n">
+      <c r="E15" s="14" t="n">
+        <v>250</v>
+      </c>
+      <c r="F15" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="14" t="n">
         <v>80</v>
       </c>
-      <c r="H15" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="3">
-        <f>SUM(D15:H15)</f>
-        <v/>
-      </c>
-      <c r="J15" s="9">
-        <f>J14+C15-I15</f>
+      <c r="H15" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="14">
+        <f>SUM(D15:G15)</f>
+        <v/>
+      </c>
+      <c r="K15" s="15">
+        <f>SUM(D15:I15)</f>
+        <v/>
+      </c>
+      <c r="L15" s="15">
+        <f>L14+C15-K15</f>
         <v/>
       </c>
     </row>
@@ -1002,15 +1111,22 @@
       <c r="G16" s="3" t="n">
         <v>80</v>
       </c>
-      <c r="H16" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" s="3">
-        <f>SUM(D16:H16)</f>
-        <v/>
-      </c>
-      <c r="J16" s="9">
-        <f>J15+C16-I16</f>
+      <c r="H16" s="10" t="n">
+        <v>150</v>
+      </c>
+      <c r="I16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="3">
+        <f>SUM(D16:G16)</f>
+        <v/>
+      </c>
+      <c r="K16" s="9">
+        <f>SUM(D16:I16)</f>
+        <v/>
+      </c>
+      <c r="L16" s="9">
+        <f>L15+C16-K16</f>
         <v/>
       </c>
     </row>
@@ -1038,51 +1154,65 @@
       <c r="G17" s="3" t="n">
         <v>80</v>
       </c>
-      <c r="H17" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" s="3">
-        <f>SUM(D17:H17)</f>
-        <v/>
-      </c>
-      <c r="J17" s="9">
-        <f>J16+C17-I17</f>
+      <c r="H17" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="3">
+        <f>SUM(D17:G17)</f>
+        <v/>
+      </c>
+      <c r="K17" s="9">
+        <f>SUM(D17:I17)</f>
+        <v/>
+      </c>
+      <c r="L17" s="9">
+        <f>L16+C17-K17</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="n">
+      <c r="A18" s="12" t="n">
         <v>12</v>
       </c>
-      <c r="B18" s="4">
+      <c r="B18" s="13">
         <f>DATE(YEAR(B6), MONTH(B6)+12, 1)</f>
         <v/>
       </c>
-      <c r="C18" s="3">
-        <f>Configuration!B7*2</f>
-        <v/>
-      </c>
-      <c r="D18" s="3" t="n">
+      <c r="C18" s="14">
+        <f>Configuration!B7*2</f>
+        <v/>
+      </c>
+      <c r="D18" s="14" t="n">
         <v>320</v>
       </c>
-      <c r="E18" s="3" t="n">
-        <v>250</v>
-      </c>
-      <c r="F18" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" s="3">
-        <f>SUM(D18:H18)</f>
-        <v/>
-      </c>
-      <c r="J18" s="9">
-        <f>J17+C18-I18</f>
+      <c r="E18" s="14" t="n">
+        <v>250</v>
+      </c>
+      <c r="F18" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="14">
+        <f>SUM(D18:G18)</f>
+        <v/>
+      </c>
+      <c r="K18" s="15">
+        <f>SUM(D18:I18)</f>
+        <v/>
+      </c>
+      <c r="L18" s="15">
+        <f>L17+C18-K18</f>
         <v/>
       </c>
     </row>
@@ -1110,15 +1240,22 @@
       <c r="G19" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H19" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" s="3">
-        <f>SUM(D19:H19)</f>
-        <v/>
-      </c>
-      <c r="J19" s="9">
-        <f>J18+C19-I19</f>
+      <c r="H19" s="10" t="n">
+        <v>750</v>
+      </c>
+      <c r="I19" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="3">
+        <f>SUM(D19:G19)</f>
+        <v/>
+      </c>
+      <c r="K19" s="9">
+        <f>SUM(D19:I19)</f>
+        <v/>
+      </c>
+      <c r="L19" s="9">
+        <f>L18+C19-K19</f>
         <v/>
       </c>
     </row>
@@ -1146,51 +1283,65 @@
       <c r="G20" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H20" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I20" s="3">
-        <f>SUM(D20:H20)</f>
-        <v/>
-      </c>
-      <c r="J20" s="9">
-        <f>J19+C20-I20</f>
+      <c r="H20" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" s="3">
+        <f>SUM(D20:G20)</f>
+        <v/>
+      </c>
+      <c r="K20" s="9">
+        <f>SUM(D20:I20)</f>
+        <v/>
+      </c>
+      <c r="L20" s="9">
+        <f>L19+C20-K20</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="n">
+      <c r="A21" s="12" t="n">
         <v>15</v>
       </c>
-      <c r="B21" s="4">
+      <c r="B21" s="13">
         <f>DATE(YEAR(B6), MONTH(B6)+15, 1)</f>
         <v/>
       </c>
-      <c r="C21" s="3">
-        <f>Configuration!B7*2</f>
-        <v/>
-      </c>
-      <c r="D21" s="3" t="n">
+      <c r="C21" s="14">
+        <f>Configuration!B7*2</f>
+        <v/>
+      </c>
+      <c r="D21" s="14" t="n">
         <v>320</v>
       </c>
-      <c r="E21" s="3" t="n">
-        <v>250</v>
-      </c>
-      <c r="F21" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H21" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I21" s="3">
-        <f>SUM(D21:H21)</f>
-        <v/>
-      </c>
-      <c r="J21" s="9">
-        <f>J20+C21-I21</f>
+      <c r="E21" s="14" t="n">
+        <v>250</v>
+      </c>
+      <c r="F21" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" s="14">
+        <f>SUM(D21:G21)</f>
+        <v/>
+      </c>
+      <c r="K21" s="15">
+        <f>SUM(D21:I21)</f>
+        <v/>
+      </c>
+      <c r="L21" s="15">
+        <f>L20+C21-K21</f>
         <v/>
       </c>
     </row>
@@ -1218,15 +1369,22 @@
       <c r="G22" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H22" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I22" s="3">
-        <f>SUM(D22:H22)</f>
-        <v/>
-      </c>
-      <c r="J22" s="9">
-        <f>J21+C22-I22</f>
+      <c r="H22" s="10" t="n">
+        <v>2550</v>
+      </c>
+      <c r="I22" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" s="3">
+        <f>SUM(D22:G22)</f>
+        <v/>
+      </c>
+      <c r="K22" s="9">
+        <f>SUM(D22:I22)</f>
+        <v/>
+      </c>
+      <c r="L22" s="9">
+        <f>L21+C22-K22</f>
         <v/>
       </c>
     </row>
@@ -1254,51 +1412,65 @@
       <c r="G23" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H23" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" s="3">
-        <f>SUM(D23:H23)</f>
-        <v/>
-      </c>
-      <c r="J23" s="9">
-        <f>J22+C23-I23</f>
+      <c r="H23" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" s="3">
+        <f>SUM(D23:G23)</f>
+        <v/>
+      </c>
+      <c r="K23" s="9">
+        <f>SUM(D23:I23)</f>
+        <v/>
+      </c>
+      <c r="L23" s="9">
+        <f>L22+C23-K23</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="n">
+      <c r="A24" s="12" t="n">
         <v>18</v>
       </c>
-      <c r="B24" s="4">
+      <c r="B24" s="13">
         <f>DATE(YEAR(B6), MONTH(B6)+18, 1)</f>
         <v/>
       </c>
-      <c r="C24" s="3">
-        <f>Configuration!B7*2</f>
-        <v/>
-      </c>
-      <c r="D24" s="3" t="n">
+      <c r="C24" s="14">
+        <f>Configuration!B7*2</f>
+        <v/>
+      </c>
+      <c r="D24" s="14" t="n">
         <v>320</v>
       </c>
-      <c r="E24" s="3" t="n">
-        <v>250</v>
-      </c>
-      <c r="F24" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" s="3">
-        <f>SUM(D24:H24)</f>
-        <v/>
-      </c>
-      <c r="J24" s="9">
-        <f>J23+C24-I24</f>
+      <c r="E24" s="14" t="n">
+        <v>250</v>
+      </c>
+      <c r="F24" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="14">
+        <f>SUM(D24:G24)</f>
+        <v/>
+      </c>
+      <c r="K24" s="15">
+        <f>SUM(D24:I24)</f>
+        <v/>
+      </c>
+      <c r="L24" s="15">
+        <f>L23+C24-K24</f>
         <v/>
       </c>
     </row>
@@ -1326,15 +1498,22 @@
       <c r="G25" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H25" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I25" s="3">
-        <f>SUM(D25:H25)</f>
-        <v/>
-      </c>
-      <c r="J25" s="9">
-        <f>J24+C25-I25</f>
+      <c r="H25" s="10" t="n">
+        <v>750</v>
+      </c>
+      <c r="I25" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="3">
+        <f>SUM(D25:G25)</f>
+        <v/>
+      </c>
+      <c r="K25" s="9">
+        <f>SUM(D25:I25)</f>
+        <v/>
+      </c>
+      <c r="L25" s="9">
+        <f>L24+C25-K25</f>
         <v/>
       </c>
     </row>
@@ -1362,51 +1541,65 @@
       <c r="G26" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H26" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I26" s="3">
-        <f>SUM(D26:H26)</f>
-        <v/>
-      </c>
-      <c r="J26" s="9">
-        <f>J25+C26-I26</f>
+      <c r="H26" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" s="3">
+        <f>SUM(D26:G26)</f>
+        <v/>
+      </c>
+      <c r="K26" s="9">
+        <f>SUM(D26:I26)</f>
+        <v/>
+      </c>
+      <c r="L26" s="9">
+        <f>L25+C26-K26</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="n">
+      <c r="A27" s="12" t="n">
         <v>21</v>
       </c>
-      <c r="B27" s="4">
+      <c r="B27" s="13">
         <f>DATE(YEAR(B6), MONTH(B6)+21, 1)</f>
         <v/>
       </c>
-      <c r="C27" s="3">
-        <f>Configuration!B7*2</f>
-        <v/>
-      </c>
-      <c r="D27" s="3" t="n">
+      <c r="C27" s="14">
+        <f>Configuration!B7*2</f>
+        <v/>
+      </c>
+      <c r="D27" s="14" t="n">
         <v>320</v>
       </c>
-      <c r="E27" s="3" t="n">
-        <v>250</v>
-      </c>
-      <c r="F27" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G27" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H27" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I27" s="3">
-        <f>SUM(D27:H27)</f>
-        <v/>
-      </c>
-      <c r="J27" s="9">
-        <f>J26+C27-I27</f>
+      <c r="E27" s="14" t="n">
+        <v>250</v>
+      </c>
+      <c r="F27" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="14">
+        <f>SUM(D27:G27)</f>
+        <v/>
+      </c>
+      <c r="K27" s="15">
+        <f>SUM(D27:I27)</f>
+        <v/>
+      </c>
+      <c r="L27" s="15">
+        <f>L26+C27-K27</f>
         <v/>
       </c>
     </row>
@@ -1434,15 +1627,22 @@
       <c r="G28" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H28" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I28" s="3">
-        <f>SUM(D28:H28)</f>
-        <v/>
-      </c>
-      <c r="J28" s="9">
-        <f>J27+C28-I28</f>
+      <c r="H28" s="10" t="n">
+        <v>150</v>
+      </c>
+      <c r="I28" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="3">
+        <f>SUM(D28:G28)</f>
+        <v/>
+      </c>
+      <c r="K28" s="9">
+        <f>SUM(D28:I28)</f>
+        <v/>
+      </c>
+      <c r="L28" s="9">
+        <f>L27+C28-K28</f>
         <v/>
       </c>
     </row>
@@ -1470,90 +1670,644 @@
       <c r="G29" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H29" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I29" s="3">
-        <f>SUM(D29:H29)</f>
-        <v/>
-      </c>
-      <c r="J29" s="9">
-        <f>J28+C29-I29</f>
+      <c r="H29" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" s="3">
+        <f>SUM(D29:G29)</f>
+        <v/>
+      </c>
+      <c r="K29" s="9">
+        <f>SUM(D29:I29)</f>
+        <v/>
+      </c>
+      <c r="L29" s="9">
+        <f>L28+C29-K29</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="n">
+      <c r="A30" s="12" t="n">
         <v>24</v>
       </c>
-      <c r="B30" s="4">
+      <c r="B30" s="13">
         <f>DATE(YEAR(B6), MONTH(B6)+24, 1)</f>
         <v/>
       </c>
-      <c r="C30" s="3">
-        <f>Configuration!B7*2</f>
-        <v/>
-      </c>
-      <c r="D30" s="3" t="n">
+      <c r="C30" s="14">
+        <f>Configuration!B7*2</f>
+        <v/>
+      </c>
+      <c r="D30" s="14" t="n">
         <v>320</v>
       </c>
-      <c r="E30" s="3" t="n">
-        <v>250</v>
-      </c>
-      <c r="F30" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G30" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H30" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I30" s="3">
-        <f>SUM(D30:H30)</f>
-        <v/>
-      </c>
-      <c r="J30" s="9">
-        <f>J29+C30-I30</f>
+      <c r="E30" s="14" t="n">
+        <v>250</v>
+      </c>
+      <c r="F30" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" s="14">
+        <f>SUM(D30:G30)</f>
+        <v/>
+      </c>
+      <c r="K30" s="15">
+        <f>SUM(D30:I30)</f>
+        <v/>
+      </c>
+      <c r="L30" s="15">
+        <f>L29+C30-K30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>25</v>
+      </c>
+      <c r="B31" s="4">
+        <f>DATE(YEAR(B6), MONTH(B6)+25, 1)</f>
+        <v/>
+      </c>
+      <c r="C31" s="3">
+        <f>Configuration!B7*2</f>
+        <v/>
+      </c>
+      <c r="D31" s="3" t="n">
+        <v>320</v>
+      </c>
+      <c r="E31" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="F31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="10" t="n">
+        <v>750</v>
+      </c>
+      <c r="I31" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" s="3">
+        <f>SUM(D31:G31)</f>
+        <v/>
+      </c>
+      <c r="K31" s="9">
+        <f>SUM(D31:I31)</f>
+        <v/>
+      </c>
+      <c r="L31" s="9">
+        <f>L30+C31-K31</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="A32" t="n">
+        <v>26</v>
+      </c>
+      <c r="B32" s="4">
+        <f>DATE(YEAR(B6), MONTH(B6)+26, 1)</f>
+        <v/>
+      </c>
+      <c r="C32" s="3">
+        <f>Configuration!B7*2</f>
+        <v/>
+      </c>
+      <c r="D32" s="3" t="n">
+        <v>320</v>
+      </c>
+      <c r="E32" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="F32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J32" s="3">
+        <f>SUM(D32:G32)</f>
+        <v/>
+      </c>
+      <c r="K32" s="9">
+        <f>SUM(D32:I32)</f>
+        <v/>
+      </c>
+      <c r="L32" s="9">
+        <f>L31+C32-K32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="n">
+        <v>27</v>
+      </c>
+      <c r="B33" s="13">
+        <f>DATE(YEAR(B6), MONTH(B6)+27, 1)</f>
+        <v/>
+      </c>
+      <c r="C33" s="14">
+        <f>Configuration!B7*2</f>
+        <v/>
+      </c>
+      <c r="D33" s="14" t="n">
+        <v>320</v>
+      </c>
+      <c r="E33" s="14" t="n">
+        <v>250</v>
+      </c>
+      <c r="F33" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" s="14">
+        <f>SUM(D33:G33)</f>
+        <v/>
+      </c>
+      <c r="K33" s="15">
+        <f>SUM(D33:I33)</f>
+        <v/>
+      </c>
+      <c r="L33" s="15">
+        <f>L32+C33-K33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>28</v>
+      </c>
+      <c r="B34" s="4">
+        <f>DATE(YEAR(B6), MONTH(B6)+28, 1)</f>
+        <v/>
+      </c>
+      <c r="C34" s="3">
+        <f>Configuration!B7*2</f>
+        <v/>
+      </c>
+      <c r="D34" s="3" t="n">
+        <v>320</v>
+      </c>
+      <c r="E34" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="F34" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="10" t="n">
+        <v>2550</v>
+      </c>
+      <c r="I34" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" s="3">
+        <f>SUM(D34:G34)</f>
+        <v/>
+      </c>
+      <c r="K34" s="9">
+        <f>SUM(D34:I34)</f>
+        <v/>
+      </c>
+      <c r="L34" s="9">
+        <f>L33+C34-K34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>29</v>
+      </c>
+      <c r="B35" s="4">
+        <f>DATE(YEAR(B6), MONTH(B6)+29, 1)</f>
+        <v/>
+      </c>
+      <c r="C35" s="3">
+        <f>Configuration!B7*2</f>
+        <v/>
+      </c>
+      <c r="D35" s="3" t="n">
+        <v>320</v>
+      </c>
+      <c r="E35" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="F35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I35" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" s="3">
+        <f>SUM(D35:G35)</f>
+        <v/>
+      </c>
+      <c r="K35" s="9">
+        <f>SUM(D35:I35)</f>
+        <v/>
+      </c>
+      <c r="L35" s="9">
+        <f>L34+C35-K35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="12" t="n">
+        <v>30</v>
+      </c>
+      <c r="B36" s="13">
+        <f>DATE(YEAR(B6), MONTH(B6)+30, 1)</f>
+        <v/>
+      </c>
+      <c r="C36" s="14">
+        <f>Configuration!B7*2</f>
+        <v/>
+      </c>
+      <c r="D36" s="14" t="n">
+        <v>320</v>
+      </c>
+      <c r="E36" s="14" t="n">
+        <v>250</v>
+      </c>
+      <c r="F36" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" s="14">
+        <f>SUM(D36:G36)</f>
+        <v/>
+      </c>
+      <c r="K36" s="15">
+        <f>SUM(D36:I36)</f>
+        <v/>
+      </c>
+      <c r="L36" s="15">
+        <f>L35+C36-K36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>31</v>
+      </c>
+      <c r="B37" s="4">
+        <f>DATE(YEAR(B6), MONTH(B6)+31, 1)</f>
+        <v/>
+      </c>
+      <c r="C37" s="3">
+        <f>Configuration!B7*2</f>
+        <v/>
+      </c>
+      <c r="D37" s="3" t="n">
+        <v>320</v>
+      </c>
+      <c r="E37" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="F37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" s="10" t="n">
+        <v>750</v>
+      </c>
+      <c r="I37" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" s="3">
+        <f>SUM(D37:G37)</f>
+        <v/>
+      </c>
+      <c r="K37" s="9">
+        <f>SUM(D37:I37)</f>
+        <v/>
+      </c>
+      <c r="L37" s="9">
+        <f>L36+C37-K37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>32</v>
+      </c>
+      <c r="B38" s="4">
+        <f>DATE(YEAR(B6), MONTH(B6)+32, 1)</f>
+        <v/>
+      </c>
+      <c r="C38" s="3">
+        <f>Configuration!B7*2</f>
+        <v/>
+      </c>
+      <c r="D38" s="3" t="n">
+        <v>320</v>
+      </c>
+      <c r="E38" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="F38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" s="3">
+        <f>SUM(D38:G38)</f>
+        <v/>
+      </c>
+      <c r="K38" s="9">
+        <f>SUM(D38:I38)</f>
+        <v/>
+      </c>
+      <c r="L38" s="9">
+        <f>L37+C38-K38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="12" t="n">
+        <v>33</v>
+      </c>
+      <c r="B39" s="13">
+        <f>DATE(YEAR(B6), MONTH(B6)+33, 1)</f>
+        <v/>
+      </c>
+      <c r="C39" s="14">
+        <f>Configuration!B7*2</f>
+        <v/>
+      </c>
+      <c r="D39" s="14" t="n">
+        <v>320</v>
+      </c>
+      <c r="E39" s="14" t="n">
+        <v>250</v>
+      </c>
+      <c r="F39" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" s="14">
+        <f>SUM(D39:G39)</f>
+        <v/>
+      </c>
+      <c r="K39" s="15">
+        <f>SUM(D39:I39)</f>
+        <v/>
+      </c>
+      <c r="L39" s="15">
+        <f>L38+C39-K39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>34</v>
+      </c>
+      <c r="B40" s="4">
+        <f>DATE(YEAR(B6), MONTH(B6)+34, 1)</f>
+        <v/>
+      </c>
+      <c r="C40" s="3">
+        <f>Configuration!B7*2</f>
+        <v/>
+      </c>
+      <c r="D40" s="3" t="n">
+        <v>320</v>
+      </c>
+      <c r="E40" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="F40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" s="10" t="n">
+        <v>150</v>
+      </c>
+      <c r="I40" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J40" s="3">
+        <f>SUM(D40:G40)</f>
+        <v/>
+      </c>
+      <c r="K40" s="9">
+        <f>SUM(D40:I40)</f>
+        <v/>
+      </c>
+      <c r="L40" s="9">
+        <f>L39+C40-K40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>35</v>
+      </c>
+      <c r="B41" s="4">
+        <f>DATE(YEAR(B6), MONTH(B6)+35, 1)</f>
+        <v/>
+      </c>
+      <c r="C41" s="3">
+        <f>Configuration!B7*2</f>
+        <v/>
+      </c>
+      <c r="D41" s="3" t="n">
+        <v>320</v>
+      </c>
+      <c r="E41" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="F41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" s="3">
+        <f>SUM(D41:G41)</f>
+        <v/>
+      </c>
+      <c r="K41" s="9">
+        <f>SUM(D41:I41)</f>
+        <v/>
+      </c>
+      <c r="L41" s="9">
+        <f>L40+C41-K41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="12" t="n">
+        <v>36</v>
+      </c>
+      <c r="B42" s="13">
+        <f>DATE(YEAR(B6), MONTH(B6)+36, 1)</f>
+        <v/>
+      </c>
+      <c r="C42" s="14">
+        <f>Configuration!B7*2</f>
+        <v/>
+      </c>
+      <c r="D42" s="14" t="n">
+        <v>320</v>
+      </c>
+      <c r="E42" s="14" t="n">
+        <v>250</v>
+      </c>
+      <c r="F42" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J42" s="14">
+        <f>SUM(D42:G42)</f>
+        <v/>
+      </c>
+      <c r="K42" s="15">
+        <f>SUM(D42:I42)</f>
+        <v/>
+      </c>
+      <c r="L42" s="15">
+        <f>L41+C42-K42</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>Notes:</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>• Update 'Other Expenses' column for one-time or variable expenses</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>• Recurring expense amounts are based on 'Expense History' sheet</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>• Add more columns for additional recurring expense categories as needed</t>
+    <row r="45">
+      <c r="A45" s="16" t="inlineStr">
+        <is>
+          <t>• Yellow cells (Non-Monthly): Automatically populated from Non-Monthly Expenses sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="16" t="inlineStr">
+        <is>
+          <t>• Green cells (Other Expenses): Manual entry for unexpected or one-time expenses</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="16" t="inlineStr">
+        <is>
+          <t>• Total Recurring: Sum of regular monthly expenses only (Xcel, Verizon, Lawn, Dog Walking, etc.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="16" t="inlineStr">
+        <is>
+          <t>• Total Expenses: Includes recurring + non-monthly + other expenses</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="16" t="inlineStr">
+        <is>
+          <t>• Extend the projection by copying the formulas down to add more months</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="16" t="inlineStr">
+        <is>
+          <t>• Update recurring expense amounts in columns D-G when rates change</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A3:J3"/>
-    <mergeCell ref="A34:J34"/>
-    <mergeCell ref="A35:J35"/>
-    <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A33:J33"/>
+  <mergeCells count="9">
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A49:L49"/>
+    <mergeCell ref="A47:L47"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A45:L45"/>
+    <mergeCell ref="A46:L46"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="A50:L50"/>
+    <mergeCell ref="A48:L48"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1597,27 +2351,27 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Expense Name</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>Effective Date</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="C5" s="17" t="inlineStr">
         <is>
           <t>Monthly Amount</t>
         </is>
       </c>
-      <c r="D5" s="10" t="inlineStr">
+      <c r="D5" s="17" t="inlineStr">
         <is>
           <t>Frequency</t>
         </is>
       </c>
-      <c r="E5" s="10" t="inlineStr">
+      <c r="E5" s="17" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -1875,7 +2629,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="11" t="inlineStr">
+      <c r="A21" s="16" t="inlineStr">
         <is>
           <t>Frequency options: Monthly, Quarterly, Semi-Annual, Annual</t>
         </is>
@@ -1890,4 +2644,279 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Non-Monthly &amp; One-Time Expenses</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Track quarterly, semi-annual, annual, and one-time expenses here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>These expenses will be included in your projection at the appropriate times.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>Expense Name</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="C5" s="18" t="inlineStr">
+        <is>
+          <t>Frequency</t>
+        </is>
+      </c>
+      <c r="D5" s="18" t="inlineStr">
+        <is>
+          <t>First Payment Date</t>
+        </is>
+      </c>
+      <c r="E5" s="18" t="inlineStr">
+        <is>
+          <t>Last Payment Date</t>
+        </is>
+      </c>
+      <c r="F5" s="18" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>HOA Fees</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Quarterly</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>46023</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>47118</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Paid in Jan, Apr, Jul, Oct</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Car Insurance</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>600</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Semi-Annual</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>46023</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>47118</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Paid in Jan and Jul</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Property Tax</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>2400</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>46113</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>47118</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Paid once per year in April</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Amazon Prime</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>139</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>46082</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>47118</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Annual subscription</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Holiday Gifts</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>800</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>46357</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>47118</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>December shopping</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Car Registration</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>180</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>46174</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>47118</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Renew in June</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Frequency Guide:</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>• Quarterly: Every 3 months (4 times per year)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>• Semi-Annual: Every 6 months (2 times per year)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>• Annual: Once per year</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>• One-Time: Single occurrence (enter same date for First and Last Payment Date)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A15:F15"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>